<commit_message>
Update payroll data and dashboard template
</commit_message>
<xml_diff>
--- a/data/PAYROLL.xlsx
+++ b/data/PAYROLL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Python\hr_dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CBF01E6-7F53-41FB-9C35-06177A6331B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF847203-46F4-4DBB-B96C-11D0A87CB98F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -68,6 +68,9 @@
     <t>SALES REP</t>
   </si>
   <si>
+    <t>Started working on 27th july. Took off 2nd Aug. need to deduct next pay 08/20</t>
+  </si>
+  <si>
     <t>Kamran</t>
   </si>
   <si>
@@ -84,6 +87,9 @@
   </si>
   <si>
     <t>Jeemy</t>
+  </si>
+  <si>
+    <t>Started working on 23th july. Took off 2nd Aug. need to deduct next pay 08/20</t>
   </si>
   <si>
     <t>Jeremy</t>
@@ -108,12 +114,6 @@
   </si>
   <si>
     <t>GRAND TOTAL</t>
-  </si>
-  <si>
-    <t>Started working on 27th july. Took off 2nd Aug. need to deduct next pay 08/20</t>
-  </si>
-  <si>
-    <t>Started working on 23th july. Took off 2nd Aug. need to deduct next pay 08/20</t>
   </si>
 </sst>
 </file>
@@ -762,7 +762,7 @@
         <v>46239</v>
       </c>
       <c r="D2" s="11">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>9</v>
@@ -774,10 +774,11 @@
         <v>10</v>
       </c>
       <c r="H2" s="6">
-        <v>822</v>
+        <f>+D2*G2</f>
+        <v>850</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
@@ -814,7 +815,7 @@
         <v>65</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F3" s="5" t="s">
         <v>10</v>
@@ -823,6 +824,7 @@
         <v>10</v>
       </c>
       <c r="H3" s="6">
+        <f t="shared" ref="H3:H14" si="0">+D3*G3</f>
         <v>650</v>
       </c>
       <c r="I3" s="5"/>
@@ -861,15 +863,16 @@
         <v>75</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G4" s="10">
         <v>10</v>
       </c>
       <c r="H4" s="6">
+        <f t="shared" si="0"/>
         <v>750</v>
       </c>
       <c r="I4" s="5"/>
@@ -908,15 +911,16 @@
         <v>73</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G5" s="10">
         <v>10</v>
       </c>
       <c r="H5" s="6">
+        <f t="shared" si="0"/>
         <v>730</v>
       </c>
       <c r="I5" s="5"/>
@@ -955,15 +959,16 @@
         <v>81</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6" s="10">
         <v>10</v>
       </c>
       <c r="H6" s="6">
+        <f t="shared" si="0"/>
         <v>810</v>
       </c>
       <c r="I6" s="5"/>
@@ -1002,19 +1007,20 @@
         <v>66</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G7" s="10">
         <v>10</v>
       </c>
       <c r="H7" s="6">
+        <f t="shared" si="0"/>
         <v>660</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
@@ -1051,7 +1057,7 @@
         <v>58</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>10</v>
@@ -1060,6 +1066,7 @@
         <v>10</v>
       </c>
       <c r="H8" s="6">
+        <f t="shared" si="0"/>
         <v>580</v>
       </c>
       <c r="I8" s="5"/>
@@ -1098,7 +1105,7 @@
         <v>49</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>10</v>
@@ -1107,6 +1114,7 @@
         <v>10</v>
       </c>
       <c r="H9" s="6">
+        <f t="shared" si="0"/>
         <v>490</v>
       </c>
       <c r="I9" s="5"/>
@@ -1145,7 +1153,7 @@
         <v>67</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>10</v>
@@ -1154,6 +1162,7 @@
         <v>10</v>
       </c>
       <c r="H10" s="6">
+        <f t="shared" si="0"/>
         <v>670</v>
       </c>
       <c r="I10" s="5"/>
@@ -1192,7 +1201,7 @@
         <v>69</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>10</v>
@@ -1201,6 +1210,7 @@
         <v>10</v>
       </c>
       <c r="H11" s="6">
+        <f t="shared" si="0"/>
         <v>690</v>
       </c>
       <c r="I11" s="5"/>
@@ -1239,7 +1249,7 @@
         <v>63</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>10</v>
@@ -1248,6 +1258,7 @@
         <v>10</v>
       </c>
       <c r="H12" s="6">
+        <f t="shared" si="0"/>
         <v>630</v>
       </c>
       <c r="I12" s="5"/>
@@ -1286,7 +1297,7 @@
         <v>59</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F13" s="5" t="s">
         <v>10</v>
@@ -1295,6 +1306,7 @@
         <v>10</v>
       </c>
       <c r="H13" s="6">
+        <f t="shared" si="0"/>
         <v>590</v>
       </c>
       <c r="I13" s="5"/>
@@ -1333,7 +1345,7 @@
         <v>58</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F14" s="5" t="s">
         <v>10</v>
@@ -1342,6 +1354,7 @@
         <v>10</v>
       </c>
       <c r="H14" s="6">
+        <f t="shared" si="0"/>
         <v>580</v>
       </c>
       <c r="I14" s="5"/>
@@ -1678,7 +1691,7 @@
     </row>
     <row r="25" spans="1:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="14" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -1688,7 +1701,7 @@
       <c r="G25" s="7"/>
       <c r="H25" s="8">
         <f>SUBTOTAL(9,H2:H24)</f>
-        <v>8652</v>
+        <v>8680</v>
       </c>
       <c r="I25" s="12"/>
       <c r="J25" s="3"/>

</xml_diff>